<commit_message>
Update scene sheets, lyrics, and add loop asset/test files
</commit_message>
<xml_diff>
--- a/Feuilles/Regrets.xlsx
+++ b/Feuilles/Regrets.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10914"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tanaismusic/Documents/CLIC/Feuilles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{928B07C9-0780-AF4D-A4B3-39598C1DFD5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8B848FF-387A-7148-AE68-B9F838D99FAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1600" yWindow="2240" windowWidth="28040" windowHeight="17440" xr2:uid="{2F1647A4-8C84-E14B-83BA-CB692A19D8A6}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>MES</t>
   </si>
@@ -65,9 +65,6 @@
     <t>PONT</t>
   </si>
   <si>
-    <t>REFRAIN 3</t>
-  </si>
-  <si>
     <t xml:space="preserve">COUPLET 2 </t>
   </si>
   <si>
@@ -87,6 +84,12 @@
   </si>
   <si>
     <t>LOOP</t>
+  </si>
+  <si>
+    <t>REFRAIN 3a</t>
+  </si>
+  <si>
+    <t>REFRAIN 3b</t>
   </si>
 </sst>
 </file>
@@ -475,7 +478,7 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
@@ -715,7 +718,7 @@
         <v>0</v>
       </c>
       <c r="D22" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
@@ -1120,7 +1123,7 @@
         <v>0</v>
       </c>
       <c r="D58" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
@@ -1211,7 +1214,7 @@
         <v>0</v>
       </c>
       <c r="D66" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E66">
         <v>1</v>
@@ -1305,7 +1308,7 @@
         <v>0</v>
       </c>
       <c r="D74" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E74">
         <v>1</v>
@@ -1399,7 +1402,7 @@
         <v>0</v>
       </c>
       <c r="D82" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="E82">
         <v>1</v>
@@ -1492,6 +1495,9 @@
       <c r="C90">
         <v>0</v>
       </c>
+      <c r="D90" t="s">
+        <v>16</v>
+      </c>
       <c r="E90">
         <v>1</v>
       </c>
@@ -1584,10 +1590,10 @@
         <v>0</v>
       </c>
       <c r="D98" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E98">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.2">
@@ -1677,9 +1683,6 @@
       <c r="C106">
         <v>0</v>
       </c>
-      <c r="E106">
-        <v>0</v>
-      </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A107">
@@ -1725,7 +1728,7 @@
         <v>0</v>
       </c>
       <c r="D110" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.2">

</xml_diff>